<commit_message>
memo hernoemd en stroomdiagram apart gezet
</commit_message>
<xml_diff>
--- a/zib2017-2020/mapping deprecated zibs/all-translations.xlsx
+++ b/zib2017-2020/mapping deprecated zibs/all-translations.xlsx
@@ -11,19 +11,19 @@
     <sheet name="translations" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">translations!$A$1:$L$18</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">translations!$A$1:$L$17</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="86">
   <si>
     <t>Generated file. Do not edit this workbook, edit the individual zib workbooks instead.</t>
   </si>
   <si>
-    <t>02-10-2025 18:03</t>
+    <t>07-10-2025 16:24</t>
   </si>
   <si>
     <t>ZibName 2017</t>
@@ -80,9 +80,6 @@
     <t>NL-CM:2.1.10</t>
   </si>
   <si>
-    <t>NL-CM:0.0.14</t>
-  </si>
-  <si>
     <t>NL-CM:2.1.3</t>
   </si>
   <si>
@@ -117,9 +114,6 @@
   </si>
   <si>
     <t>VerificatieDatum</t>
-  </si>
-  <si>
-    <t>DatumTijd (Basiselementen)</t>
   </si>
   <si>
     <t>Behandeling</t>
@@ -254,9 +248,6 @@
 Zie stroomdiagram Verificatie voor de situatie met meerdere voorkomens van Verificatie.</t>
   </si>
   <si>
-    <t>zie Verificatiedatum</t>
-  </si>
-  <si>
     <t>overnemen</t>
   </si>
   <si>
@@ -266,6 +257,9 @@
   </si>
   <si>
     <t>overnemen, voorafgegaan door de tekst "Ja, maar met beperkingen: "</t>
+  </si>
+  <si>
+    <t>zie Verificatiedatum</t>
   </si>
   <si>
     <t>overnemen
@@ -704,7 +698,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L18"/>
+  <dimension ref="A1:L17"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="40.7109375" customWidth="1"/>
@@ -763,16 +757,16 @@
         <v>14</v>
       </c>
       <c r="E2" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="F2" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="G2" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="H2" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
     </row>
     <row r="3" spans="1:12">
@@ -783,16 +777,16 @@
         <v>16</v>
       </c>
       <c r="C3" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="H3" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="J3" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="K3" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="4" spans="1:12">
@@ -803,13 +797,13 @@
         <v>17</v>
       </c>
       <c r="C4" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="H4" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="K4" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="5" spans="1:12">
@@ -820,28 +814,28 @@
         <v>18</v>
       </c>
       <c r="C5" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D5" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="E5" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="F5" t="s">
+        <v>46</v>
+      </c>
+      <c r="G5" t="s">
         <v>48</v>
       </c>
-      <c r="G5" t="s">
-        <v>50</v>
-      </c>
       <c r="H5" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="J5" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="K5" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
     </row>
     <row r="6" spans="1:12">
@@ -852,25 +846,25 @@
         <v>19</v>
       </c>
       <c r="C6" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E6" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="F6" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="G6" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="H6" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="J6" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="K6" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
     </row>
     <row r="7" spans="1:12">
@@ -881,22 +875,31 @@
         <v>20</v>
       </c>
       <c r="C7" t="s">
-        <v>33</v>
+        <v>32</v>
+      </c>
+      <c r="D7" t="s">
+        <v>42</v>
       </c>
       <c r="E7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F7" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="G7" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="H7" t="s">
-        <v>64</v>
+        <v>32</v>
+      </c>
+      <c r="I7" t="s">
+        <v>42</v>
       </c>
       <c r="J7" t="s">
-        <v>76</v>
+        <v>74</v>
+      </c>
+      <c r="K7" t="s">
+        <v>74</v>
       </c>
     </row>
     <row r="8" spans="1:12">
@@ -907,31 +910,31 @@
         <v>21</v>
       </c>
       <c r="C8" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D8" t="s">
+        <v>43</v>
+      </c>
+      <c r="E8" t="s">
         <v>44</v>
       </c>
-      <c r="E8" t="s">
-        <v>47</v>
-      </c>
       <c r="F8" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="G8" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="H8" t="s">
-        <v>34</v>
+        <v>63</v>
       </c>
       <c r="I8" t="s">
-        <v>44</v>
+        <v>70</v>
       </c>
       <c r="J8" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="K8" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
     </row>
     <row r="9" spans="1:12">
@@ -942,31 +945,25 @@
         <v>22</v>
       </c>
       <c r="C9" t="s">
-        <v>35</v>
-      </c>
-      <c r="D9" t="s">
-        <v>45</v>
+        <v>34</v>
       </c>
       <c r="E9" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="F9" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="G9" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="H9" t="s">
-        <v>65</v>
-      </c>
-      <c r="I9" t="s">
-        <v>72</v>
+        <v>64</v>
       </c>
       <c r="J9" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="K9" t="s">
-        <v>85</v>
+        <v>74</v>
       </c>
     </row>
     <row r="10" spans="1:12">
@@ -977,24 +974,21 @@
         <v>23</v>
       </c>
       <c r="C10" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E10" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="F10" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="G10" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="H10" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="J10" t="s">
-        <v>79</v>
-      </c>
-      <c r="K10" t="s">
         <v>77</v>
       </c>
     </row>
@@ -1006,22 +1000,25 @@
         <v>24</v>
       </c>
       <c r="C11" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E11" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="F11" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="G11" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="H11" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="J11" t="s">
-        <v>76</v>
+        <v>78</v>
+      </c>
+      <c r="K11" t="s">
+        <v>74</v>
       </c>
     </row>
     <row r="12" spans="1:12">
@@ -1032,25 +1029,25 @@
         <v>25</v>
       </c>
       <c r="C12" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E12" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F12" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="G12" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="H12" t="s">
-        <v>67</v>
+        <v>37</v>
       </c>
       <c r="J12" t="s">
-        <v>80</v>
+        <v>74</v>
       </c>
       <c r="K12" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
     </row>
     <row r="13" spans="1:12">
@@ -1061,148 +1058,119 @@
         <v>26</v>
       </c>
       <c r="C13" t="s">
+        <v>38</v>
+      </c>
+      <c r="E13" t="s">
+        <v>45</v>
+      </c>
+      <c r="F13" t="s">
+        <v>46</v>
+      </c>
+      <c r="G13" t="s">
+        <v>55</v>
+      </c>
+      <c r="H13" t="s">
+        <v>38</v>
+      </c>
+      <c r="J13" t="s">
+        <v>74</v>
+      </c>
+      <c r="K13" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12">
+      <c r="C14" t="s">
         <v>39</v>
       </c>
-      <c r="E13" t="s">
-        <v>47</v>
-      </c>
-      <c r="F13" t="s">
-        <v>48</v>
-      </c>
-      <c r="G13" t="s">
+      <c r="F14" t="s">
+        <v>46</v>
+      </c>
+      <c r="G14" t="s">
         <v>56</v>
       </c>
-      <c r="H13" t="s">
-        <v>39</v>
-      </c>
-      <c r="J13" t="s">
-        <v>77</v>
-      </c>
-      <c r="K13" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="14" spans="1:12">
-      <c r="A14" t="s">
-        <v>14</v>
-      </c>
-      <c r="B14" t="s">
-        <v>27</v>
-      </c>
-      <c r="C14" t="s">
-        <v>40</v>
-      </c>
-      <c r="E14" t="s">
-        <v>47</v>
-      </c>
-      <c r="F14" t="s">
-        <v>48</v>
-      </c>
-      <c r="G14" t="s">
-        <v>57</v>
-      </c>
       <c r="H14" t="s">
-        <v>40</v>
+        <v>66</v>
       </c>
       <c r="J14" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="K14" t="s">
-        <v>77</v>
+        <v>84</v>
       </c>
     </row>
     <row r="15" spans="1:12">
       <c r="C15" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="F15" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="G15" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="H15" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="J15" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="K15" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="16" spans="1:12">
       <c r="C16" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="F16" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="G16" t="s">
+        <v>58</v>
+      </c>
+      <c r="H16" t="s">
+        <v>68</v>
+      </c>
+      <c r="J16" t="s">
+        <v>79</v>
+      </c>
+      <c r="K16" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11">
+      <c r="A17" t="s">
+        <v>14</v>
+      </c>
+      <c r="B17" t="s">
+        <v>27</v>
+      </c>
+      <c r="C17" t="s">
+        <v>40</v>
+      </c>
+      <c r="E17" t="s">
+        <v>44</v>
+      </c>
+      <c r="F17" t="s">
+        <v>46</v>
+      </c>
+      <c r="G17" t="s">
         <v>59</v>
       </c>
-      <c r="H16" t="s">
+      <c r="H17" t="s">
         <v>69</v>
       </c>
-      <c r="J16" t="s">
-        <v>81</v>
-      </c>
-      <c r="K16" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="17" spans="1:11">
-      <c r="C17" t="s">
-        <v>41</v>
-      </c>
-      <c r="F17" t="s">
-        <v>48</v>
-      </c>
-      <c r="G17" t="s">
-        <v>60</v>
-      </c>
-      <c r="H17" t="s">
-        <v>70</v>
-      </c>
       <c r="J17" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="K17" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="18" spans="1:11">
-      <c r="A18" t="s">
-        <v>14</v>
-      </c>
-      <c r="B18" t="s">
-        <v>28</v>
-      </c>
-      <c r="C18" t="s">
-        <v>42</v>
-      </c>
-      <c r="E18" t="s">
-        <v>46</v>
-      </c>
-      <c r="F18" t="s">
-        <v>48</v>
-      </c>
-      <c r="G18" t="s">
-        <v>61</v>
-      </c>
-      <c r="H18" t="s">
-        <v>71</v>
-      </c>
-      <c r="J18" t="s">
-        <v>82</v>
-      </c>
-      <c r="K18" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L18"/>
-  <conditionalFormatting sqref="E2:E18">
+  <autoFilter ref="A1:L17"/>
+  <conditionalFormatting sqref="E2:E17">
     <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
       <formula>"groen: geen wijzigingen"</formula>
     </cfRule>

</xml_diff>